<commit_message>
Inflow workbook: no rows after today; guard test
The inflow workbook carried 66 placeholder rows (monthly means) up to 2026-12-21, months in the future. They are
removed (file now ends today; 108 imputed climatology days after the last real day, 2026-06-30). The data
summaries of the plant inputs are refreshed. New test: no PV or inflow workbook holds a day after today.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/phase_2_da_day_ahead_bidding/da_price_pv_inflow_forecasting/inflow_training_data_from_2015.xlsx
+++ b/phase_2_da_day_ahead_bidding/da_price_pv_inflow_forecasting/inflow_training_data_from_2015.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4374"/>
+  <dimension ref="A1:C4308"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -56440,864 +56440,6 @@
         </is>
       </c>
     </row>
-    <row r="4309">
-      <c r="A4309" s="2" t="n">
-        <v>46312</v>
-      </c>
-      <c r="B4309" t="n">
-        <v>345008.4</v>
-      </c>
-      <c r="C4309" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4310">
-      <c r="A4310" s="2" t="n">
-        <v>46313</v>
-      </c>
-      <c r="B4310" t="n">
-        <v>345008.4</v>
-      </c>
-      <c r="C4310" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4311">
-      <c r="A4311" s="2" t="n">
-        <v>46314</v>
-      </c>
-      <c r="B4311" t="n">
-        <v>345008.4</v>
-      </c>
-      <c r="C4311" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4312">
-      <c r="A4312" s="2" t="n">
-        <v>46315</v>
-      </c>
-      <c r="B4312" t="n">
-        <v>345008.4</v>
-      </c>
-      <c r="C4312" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4313">
-      <c r="A4313" s="2" t="n">
-        <v>46316</v>
-      </c>
-      <c r="B4313" t="n">
-        <v>345008.4</v>
-      </c>
-      <c r="C4313" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4314">
-      <c r="A4314" s="2" t="n">
-        <v>46317</v>
-      </c>
-      <c r="B4314" t="n">
-        <v>345008.4</v>
-      </c>
-      <c r="C4314" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4315">
-      <c r="A4315" s="2" t="n">
-        <v>46318</v>
-      </c>
-      <c r="B4315" t="n">
-        <v>345008.4</v>
-      </c>
-      <c r="C4315" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4316">
-      <c r="A4316" s="2" t="n">
-        <v>46319</v>
-      </c>
-      <c r="B4316" t="n">
-        <v>345008.4</v>
-      </c>
-      <c r="C4316" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4317">
-      <c r="A4317" s="2" t="n">
-        <v>46320</v>
-      </c>
-      <c r="B4317" t="n">
-        <v>345008.4</v>
-      </c>
-      <c r="C4317" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4318">
-      <c r="A4318" s="2" t="n">
-        <v>46321</v>
-      </c>
-      <c r="B4318" t="n">
-        <v>345008.4</v>
-      </c>
-      <c r="C4318" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4319">
-      <c r="A4319" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="B4319" t="n">
-        <v>345008.4</v>
-      </c>
-      <c r="C4319" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4320">
-      <c r="A4320" s="2" t="n">
-        <v>46323</v>
-      </c>
-      <c r="B4320" t="n">
-        <v>345008.4</v>
-      </c>
-      <c r="C4320" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4321">
-      <c r="A4321" s="2" t="n">
-        <v>46324</v>
-      </c>
-      <c r="B4321" t="n">
-        <v>345008.4</v>
-      </c>
-      <c r="C4321" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4322">
-      <c r="A4322" s="2" t="n">
-        <v>46325</v>
-      </c>
-      <c r="B4322" t="n">
-        <v>345008.4</v>
-      </c>
-      <c r="C4322" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4323">
-      <c r="A4323" s="2" t="n">
-        <v>46326</v>
-      </c>
-      <c r="B4323" t="n">
-        <v>345008.4</v>
-      </c>
-      <c r="C4323" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4324">
-      <c r="A4324" s="2" t="n">
-        <v>46327</v>
-      </c>
-      <c r="B4324" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4324" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4325">
-      <c r="A4325" s="2" t="n">
-        <v>46328</v>
-      </c>
-      <c r="B4325" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4325" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4326">
-      <c r="A4326" s="2" t="n">
-        <v>46329</v>
-      </c>
-      <c r="B4326" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4326" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4327">
-      <c r="A4327" s="2" t="n">
-        <v>46330</v>
-      </c>
-      <c r="B4327" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4327" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4328">
-      <c r="A4328" s="2" t="n">
-        <v>46331</v>
-      </c>
-      <c r="B4328" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4328" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4329">
-      <c r="A4329" s="2" t="n">
-        <v>46332</v>
-      </c>
-      <c r="B4329" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4329" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4330">
-      <c r="A4330" s="2" t="n">
-        <v>46333</v>
-      </c>
-      <c r="B4330" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4330" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4331">
-      <c r="A4331" s="2" t="n">
-        <v>46334</v>
-      </c>
-      <c r="B4331" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4331" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4332">
-      <c r="A4332" s="2" t="n">
-        <v>46335</v>
-      </c>
-      <c r="B4332" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4332" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4333">
-      <c r="A4333" s="2" t="n">
-        <v>46336</v>
-      </c>
-      <c r="B4333" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4333" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4334">
-      <c r="A4334" s="2" t="n">
-        <v>46337</v>
-      </c>
-      <c r="B4334" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4334" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4335">
-      <c r="A4335" s="2" t="n">
-        <v>46338</v>
-      </c>
-      <c r="B4335" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4335" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4336">
-      <c r="A4336" s="2" t="n">
-        <v>46339</v>
-      </c>
-      <c r="B4336" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4336" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4337">
-      <c r="A4337" s="2" t="n">
-        <v>46340</v>
-      </c>
-      <c r="B4337" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4337" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4338">
-      <c r="A4338" s="2" t="n">
-        <v>46341</v>
-      </c>
-      <c r="B4338" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4338" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4339">
-      <c r="A4339" s="2" t="n">
-        <v>46342</v>
-      </c>
-      <c r="B4339" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4339" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4340">
-      <c r="A4340" s="2" t="n">
-        <v>46343</v>
-      </c>
-      <c r="B4340" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4340" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4341">
-      <c r="A4341" s="2" t="n">
-        <v>46344</v>
-      </c>
-      <c r="B4341" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4341" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4342">
-      <c r="A4342" s="2" t="n">
-        <v>46345</v>
-      </c>
-      <c r="B4342" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4342" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4343">
-      <c r="A4343" s="2" t="n">
-        <v>46346</v>
-      </c>
-      <c r="B4343" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4343" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4344">
-      <c r="A4344" s="2" t="n">
-        <v>46347</v>
-      </c>
-      <c r="B4344" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4344" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4345">
-      <c r="A4345" s="2" t="n">
-        <v>46348</v>
-      </c>
-      <c r="B4345" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4345" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4346">
-      <c r="A4346" s="2" t="n">
-        <v>46349</v>
-      </c>
-      <c r="B4346" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4346" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4347">
-      <c r="A4347" s="2" t="n">
-        <v>46350</v>
-      </c>
-      <c r="B4347" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4347" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4348">
-      <c r="A4348" s="2" t="n">
-        <v>46351</v>
-      </c>
-      <c r="B4348" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4348" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4349">
-      <c r="A4349" s="2" t="n">
-        <v>46352</v>
-      </c>
-      <c r="B4349" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4349" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4350">
-      <c r="A4350" s="2" t="n">
-        <v>46353</v>
-      </c>
-      <c r="B4350" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4350" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4351">
-      <c r="A4351" s="2" t="n">
-        <v>46354</v>
-      </c>
-      <c r="B4351" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4351" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4352">
-      <c r="A4352" s="2" t="n">
-        <v>46355</v>
-      </c>
-      <c r="B4352" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4352" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4353">
-      <c r="A4353" s="2" t="n">
-        <v>46356</v>
-      </c>
-      <c r="B4353" t="n">
-        <v>446566.7</v>
-      </c>
-      <c r="C4353" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4354">
-      <c r="A4354" s="2" t="n">
-        <v>46357</v>
-      </c>
-      <c r="B4354" t="n">
-        <v>550213.7</v>
-      </c>
-      <c r="C4354" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4355">
-      <c r="A4355" s="2" t="n">
-        <v>46358</v>
-      </c>
-      <c r="B4355" t="n">
-        <v>550213.7</v>
-      </c>
-      <c r="C4355" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4356">
-      <c r="A4356" s="2" t="n">
-        <v>46359</v>
-      </c>
-      <c r="B4356" t="n">
-        <v>550213.7</v>
-      </c>
-      <c r="C4356" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4357">
-      <c r="A4357" s="2" t="n">
-        <v>46360</v>
-      </c>
-      <c r="B4357" t="n">
-        <v>550213.7</v>
-      </c>
-      <c r="C4357" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4358">
-      <c r="A4358" s="2" t="n">
-        <v>46361</v>
-      </c>
-      <c r="B4358" t="n">
-        <v>550213.7</v>
-      </c>
-      <c r="C4358" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4359">
-      <c r="A4359" s="2" t="n">
-        <v>46362</v>
-      </c>
-      <c r="B4359" t="n">
-        <v>550213.7</v>
-      </c>
-      <c r="C4359" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4360">
-      <c r="A4360" s="2" t="n">
-        <v>46363</v>
-      </c>
-      <c r="B4360" t="n">
-        <v>550213.7</v>
-      </c>
-      <c r="C4360" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4361">
-      <c r="A4361" s="2" t="n">
-        <v>46364</v>
-      </c>
-      <c r="B4361" t="n">
-        <v>550213.7</v>
-      </c>
-      <c r="C4361" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4362">
-      <c r="A4362" s="2" t="n">
-        <v>46365</v>
-      </c>
-      <c r="B4362" t="n">
-        <v>550213.7</v>
-      </c>
-      <c r="C4362" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4363">
-      <c r="A4363" s="2" t="n">
-        <v>46366</v>
-      </c>
-      <c r="B4363" t="n">
-        <v>550213.7</v>
-      </c>
-      <c r="C4363" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4364">
-      <c r="A4364" s="2" t="n">
-        <v>46367</v>
-      </c>
-      <c r="B4364" t="n">
-        <v>550213.7</v>
-      </c>
-      <c r="C4364" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4365">
-      <c r="A4365" s="2" t="n">
-        <v>46368</v>
-      </c>
-      <c r="B4365" t="n">
-        <v>550213.7</v>
-      </c>
-      <c r="C4365" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4366">
-      <c r="A4366" s="2" t="n">
-        <v>46369</v>
-      </c>
-      <c r="B4366" t="n">
-        <v>550213.7</v>
-      </c>
-      <c r="C4366" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4367">
-      <c r="A4367" s="2" t="n">
-        <v>46370</v>
-      </c>
-      <c r="B4367" t="n">
-        <v>550213.7</v>
-      </c>
-      <c r="C4367" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4368">
-      <c r="A4368" s="2" t="n">
-        <v>46371</v>
-      </c>
-      <c r="B4368" t="n">
-        <v>550213.7</v>
-      </c>
-      <c r="C4368" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4369">
-      <c r="A4369" s="2" t="n">
-        <v>46372</v>
-      </c>
-      <c r="B4369" t="n">
-        <v>550213.7</v>
-      </c>
-      <c r="C4369" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4370">
-      <c r="A4370" s="2" t="n">
-        <v>46373</v>
-      </c>
-      <c r="B4370" t="n">
-        <v>550213.7</v>
-      </c>
-      <c r="C4370" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4371">
-      <c r="A4371" s="2" t="n">
-        <v>46374</v>
-      </c>
-      <c r="B4371" t="n">
-        <v>550213.7</v>
-      </c>
-      <c r="C4371" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4372">
-      <c r="A4372" s="2" t="n">
-        <v>46375</v>
-      </c>
-      <c r="B4372" t="n">
-        <v>550213.7</v>
-      </c>
-      <c r="C4372" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4373">
-      <c r="A4373" s="2" t="n">
-        <v>46376</v>
-      </c>
-      <c r="B4373" t="n">
-        <v>550213.7</v>
-      </c>
-      <c r="C4373" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4374">
-      <c r="A4374" s="2" t="n">
-        <v>46377</v>
-      </c>
-      <c r="B4374" t="n">
-        <v>550213.7</v>
-      </c>
-      <c r="C4374" t="inlineStr">
-        <is>
-          <t>Alqueva Reservoir Inflow - Monthly Climatology (gap-fill)</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>